<commit_message>
FIXED: Tutorial grid layout change && NPC fruit icon removed
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Tutorial_String_Data.xlsx
+++ b/Assets/Internationalization/Tutorial_String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C390E5-7990-467D-A2B1-0579AA4016E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75061183-5F41-4C2F-977D-186CD66C9224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="615" windowWidth="31800" windowHeight="20985" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
@@ -167,9 +167,6 @@
     <t>现在商品有点贵。\n不如先买个盲盒碰碰运气？</t>
   </si>
   <si>
-    <t>获得了 2 个自选水果。\n点击亮着的水果图标，挑你想要的吧。</t>
-  </si>
-  <si>
     <t>现在还没有升级券呢。\n先努力完成委托，在商店里买 1 张吧。</t>
   </si>
   <si>
@@ -431,6 +428,10 @@
   </si>
   <si>
     <t>确定要跳过教程吗？</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>获得了 2 个自选水果。\n点击亮着的水果图标，挑选想要的吧。</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1428,7 +1429,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>
@@ -1439,7 +1440,7 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
         <v>36</v>
@@ -1447,24 +1448,24 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" t="s">
         <v>127</v>
-      </c>
-      <c r="B4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C4" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B5" t="s">
         <v>130</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>131</v>
-      </c>
-      <c r="C5" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1472,10 +1473,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1483,7 +1484,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>40</v>
@@ -1494,7 +1495,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>41</v>
@@ -1505,15 +1506,15 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1523,7 +1524,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>42</v>
@@ -1534,7 +1535,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>38</v>
@@ -1561,10 +1562,10 @@
         <v>9</v>
       </c>
       <c r="B17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1572,7 +1573,7 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>37</v>
@@ -1583,7 +1584,7 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>43</v>
@@ -1598,7 +1599,7 @@
         <v>12</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>39</v>
@@ -1613,10 +1614,10 @@
         <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1624,10 +1625,10 @@
         <v>14</v>
       </c>
       <c r="B24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1635,10 +1636,10 @@
         <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1658,10 +1659,10 @@
         <v>16</v>
       </c>
       <c r="B29" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1669,10 +1670,10 @@
         <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1680,29 +1681,29 @@
         <v>18</v>
       </c>
       <c r="B31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" t="s">
         <v>82</v>
       </c>
-      <c r="B32" t="s">
-        <v>83</v>
-      </c>
       <c r="C32" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B33" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>44</v>
@@ -1717,7 +1718,7 @@
         <v>19</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>45</v>
@@ -1728,7 +1729,7 @@
         <v>20</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>46</v>
@@ -1739,10 +1740,10 @@
         <v>21</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>47</v>
+        <v>132</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1758,10 +1759,10 @@
         <v>22</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1769,10 +1770,10 @@
         <v>23</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1780,10 +1781,10 @@
         <v>27</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1791,10 +1792,10 @@
         <v>28</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1802,10 +1803,10 @@
         <v>29</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
@@ -1813,10 +1814,10 @@
         <v>30</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="14.25" customHeight="1">
@@ -1824,10 +1825,10 @@
         <v>31</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="14.25" customHeight="1">
@@ -1835,10 +1836,10 @@
         <v>32</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1846,10 +1847,10 @@
         <v>33</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1857,87 +1858,87 @@
         <v>34</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="28.5">
       <c r="A50" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="C50" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="C51" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="28.5">
       <c r="A52" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="C52" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="28.5">
       <c r="A53" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="C53" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="28.5">
       <c r="A54" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="C54" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="28.5">
       <c r="A55" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="C55" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="28.5">
       <c r="A56" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="C56" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1945,10 +1946,10 @@
         <v>35</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: Tutorial Shop Pool & Display_text using ratio
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Tutorial_String_Data.xlsx
+++ b/Assets/Internationalization/Tutorial_String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75061183-5F41-4C2F-977D-186CD66C9224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EBD6534-A3FC-469F-869E-DEF132C050D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="615" windowWidth="31800" windowHeight="20985" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
@@ -333,25 +333,10 @@
     <t>Manual refresh refills to 3 uses daily at 00:00.</t>
   </si>
   <si>
-    <t>手动刷新次数会在每日00:00重置为 3 次。</t>
-  </si>
-  <si>
     <t>TUTORIAL_UPGRADE_11</t>
   </si>
   <si>
-    <t>Please visit the shop again and buy the Shopping Cart.\nIf it isn’t available, try the manual refresh you just unlocked,\nor wait for a restock.</t>
-  </si>
-  <si>
-    <t>请再次拜访商店，买下 购物车 吧。\n如果目前没有上架的话，试试刚解锁的手动刷新，\n或者打发一会儿时间吧。</t>
-  </si>
-  <si>
     <t>TUTORIAL_POINTS_1</t>
-  </si>
-  <si>
-    <t>The Shopping Cart is a rare item,\nand provides 5 Shop Pts.</t>
-  </si>
-  <si>
-    <t>买到的 购物车 稀有度较高，可以提供 5 点商店点数。</t>
   </si>
   <si>
     <t>TUTORIAL_POINTS_2</t>
@@ -433,6 +418,22 @@
   <si>
     <t>获得了 2 个自选水果。\n点击亮着的水果图标，挑选想要的吧。</t>
     <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>手动刷新次数会在每日00:00重置为 3 次。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Please visit the shop again and buy the [font_size=40][color=#94b757]Balance[/color][/font_size].\nIf it isn’t available, try the manual refresh you just unlocked.</t>
+  </si>
+  <si>
+    <t>请再次拜访商店，买下 [font_size=40][color=#94b757]天平[/color][/font_size] 吧。\n如果目前没有上架的话，试试刚解锁的手动刷新吧。</t>
+  </si>
+  <si>
+    <t>The [font_size=40][color=#94b757]天平[/color][/font_size] provides 5 Shop Pts.</t>
+  </si>
+  <si>
+    <t>买到的 [font_size=40][color=#94b757]天平[/color][/font_size] 可以提供 3 点商店点数。</t>
   </si>
 </sst>
 </file>
@@ -1448,24 +1449,24 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1743,7 +1744,7 @@
         <v>85</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1784,7 +1785,7 @@
         <v>89</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1861,84 +1862,84 @@
         <v>101</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="28.5">
       <c r="A50" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>105</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="28.5">
       <c r="A52" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="28.5">
       <c r="A53" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="28.5">
       <c r="A54" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="28.5">
       <c r="A55" s="2" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="28.5">
       <c r="A56" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1946,7 +1947,7 @@
         <v>35</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>49</v>

</xml_diff>

<commit_message>
[CHANGE]tutorial text adjustment, texts that need icon marked.
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Tutorial_String_Data.xlsx
+++ b/Assets/Internationalization/Tutorial_String_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\city_of_circling\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E987EC52-A35E-4892-AAC3-2A14A964DFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A71328-EA98-4F2C-915D-A068F8CCCD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
+    <workbookView xWindow="-38510" yWindow="1250" windowWidth="38620" windowHeight="21100" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
   <sheets>
     <sheet name="String_Data" sheetId="1" r:id="rId1"/>
@@ -146,9 +146,6 @@
     <t>add_grid()</t>
   </si>
   <si>
-    <t>Someone seems to need help.\nGo pay them a visit.</t>
-  </si>
-  <si>
     <t>TUTORIAL_NPC_11</t>
   </si>
   <si>
@@ -269,26 +266,388 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>获得了[font_size=40] 苹果 x 1[/font_size]。\n虽然不知道能用来做什么...</t>
-  </si>
-  <si>
-    <t>似乎有人需要帮助。\n去拜访看看吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>还差[font_size=40] 葡萄 x 1[/font_size] 就能完成委托。</t>
-  </si>
-  <si>
     <t>抽到了需要的水果。\n现在回去提交吧。</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>“我需要[font_size=40] 苹果 x 1[/font_size] 和[font_size=40] 葡萄 x 1[/font_size]，拜托了！”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>不同于[font_size=40] 接受任务[/font_size]，\n</t>
+    <t>"可以麻烦帮我传个信给长颈鹿吗？拜托了！”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>获得了[font_size=40] 自选水果 x 2[/font_size]。\n点击闪烁的水果图标，挑选想要的吧。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>有些升级项可以反复购买，等级和效果随之提升。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>商店会在</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[color=#BC3D37]每天 00:00 [/color]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>上架随机商品，同时重置3次手动刷新次数。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>提升各类点数可以增加冒险成功率。\n不过需要四种点数共同作用，效果才会显著哦。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>四类点数道具会在对应的商店出售。\n目前没有商店能买到其他三类呢，先发放一些道具以作说明吧。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>冒险成功率提升了！\n道具准备越充分，就越能够避免冒险失败的情况。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>TUTORIAL_POINTS_7</t>
+  </si>
+  <si>
+    <t>TUTORIAL_POINTS_8</t>
+  </si>
+  <si>
+    <t>TUTORIAL_POINTS_9</t>
+  </si>
+  <si>
+    <r>
+      <t>如果</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[font_size=40] 失败 [/font_size]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>的话...就[color=#BC3D37] 一无所获 [/color]了呢。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>此外，游戏一共有[color=#BC3D37] 60 天[/color]的时间。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>花费更多时间在城里囤积道具的话，可用于出城冒险的时间则会相应减少。\n能够获得的[color=#BC3D37]  冒险得分 [/color]也会随天数降低。请注意。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>游戏的目标是获取更高的[color=#BC3D37]  冒险得分[/color]。\n因此, 在城里囤积道具的同时，努力留出更多时间用来冒险吧。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>You're ready to proceed.</t>
+  </si>
+  <si>
+    <t>Skip Tutorial</t>
+  </si>
+  <si>
+    <t>Welcome to the Tutorial.</t>
+  </si>
+  <si>
+    <t>Move your mouse along the tiles to plan a path,\nthen click the destination to confirm.</t>
+  </si>
+  <si>
+    <t>Are you sure to skip the tutorial?</t>
+  </si>
+  <si>
+    <t>Each move takes [color=#BC3D37]3 hours[/color]. Keep that in mind.</t>
+  </si>
+  <si>
+    <t>“Could you deliver a message to the Giraffe for me? Please!”</t>
+  </si>
+  <si>
+    <t>Other items are a bit pricey for now.\nHow about trying a Mystery Box instead?</t>
+  </si>
+  <si>
+    <t>Adventure success rate increased!\nThe more items you prepare, the less likely you are to fail.</t>
+  </si>
+  <si>
+    <t>Spending more time stocking up in the city means less time left for adventures.\nYour [color=#BC3D37]Adventure Score[/color] will also decrease as days pass. Keep that in mind.</t>
+  </si>
+  <si>
+    <t>The goal is to achieve a higher [color=#BC3D37]Adventure Score[/color].\nSo, stock up efficiently and leave more time for the adventure itself!</t>
+  </si>
+  <si>
+    <t>The game lasts [color=#BC3D37]60 days[/color] in total.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>准备妥当的话，就前往城门结束教程，正式开始游戏吧。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Just [font_size=40]Grapes x 1[/font_size] left to complete the quest.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Try stopping on that strange tile over there.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“Thanks for the fruit! Here are [font_size=40]Exchange Coupons x 2[/font_size].\nYou can use them at the shop.”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“I need [font_size=40]Apple x 1[/font_size] and [font_size=40]Grapes x1[/font_size], please!”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Another [font_size=40]Quest[/font_size]? Go pay them a visit.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>You got [font_size=40]Fruit of Your Choice x 2[/font_size]!\nClick the glowing fruit icons to pick the ones you want.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">There are currently two upgrades available.\nHow about buying “Shop Manual Refresh” first?  </t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Raising different types of points increases adventure success rate.\nBut only when all four types work together will the effect be significant.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>[font_size=40][color=#94b757]Balance[/color][/font_size] provides [font_size=40]3 Shop Pts[/font_size].</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>It's time to get prepared in the city for the upcoming adventure.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>You got [font_size=40]Apple x 1[/font_size]!\nNot sure what it's for yet...</t>
+  </si>
+  <si>
+    <t>The four types of items are sold at their respective shops.\nThey're not available yet, so let's give you some for demonstration.</t>
+  </si>
+  <si>
+    <t>If you [font_size=40]fail[/font_size]... you'll return [color=#BC3D37]empty-handed[/color].</t>
+  </si>
+  <si>
+    <t>Unlike [font_size=40]Accepting Quests[/font_size],\n[font_size=40]Completing Quests[/font_size] doesn't require stopping on the tile. \nPassing through will automatically deliver them.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">At the [font_size=40]Upgrade Tile[/font_size], \nyou can use [font_size=40]Upgrade Coupons[/font_size] to purchase various [font_size=40]Upgrades[/font_size].  </t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>You obtained [font_size=40]Shop Upgrade Coupon x 1[/font_size].\nGo check the shop upgrade tile.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Every day at [color=#BC3D37]00:00[/color], \nthe shop restocks with random items and also resets your 3 manual refresh uses.  </t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Some upgrades can be purchased multiple times, \nincreasing both their level and effectiveness.  </t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Now, please buy [font_size=40][color=#94b757]Balance[/color] x 1[/font_size] from the shop.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>When you're ready, \nhead to the city gate to end the tutorial and begin your adventure.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>似乎有人正在发布任务。\n去拜访看看吧。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Seems like someone's posting a quest.\nGo pay them a visit.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">“我需要[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>苹果 x 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[/font_size] 和[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>葡萄 x 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]，拜托了！”</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">还差[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>葡萄 x 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size] 就能完成任务。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">获得了[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>苹果 x 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]。\n虽然不知道能用来做什么...</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">“感谢你的水果！送你[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>交换券 x 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]，可以用来在商店购物哦。”</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">不同于[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>接受任务</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]，\n</t>
     </r>
     <r>
       <rPr>
@@ -338,75 +697,149 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>“感谢你的水果！送你[font_size=40] 交换券 x 2[/font_size]，可以用来在商店购物哦。”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>另一位似乎也有[font_size=40] 任务[/font_size]？拜访看看吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>"可以麻烦帮我传个信给长颈鹿吗？拜托了！”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>除了水果，有时也会接到传信的[font_size=40] 任务[/font_size]。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“感谢！给你[font_size=40] 交换券 x 1[/font_size]，有空的话去附近的商店看看吧。”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>商店开张，可以用交换券购物了。\n进去看看吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>其他商品有点贵。\n不如先买个盲盒碰碰运气？</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>获得了[font_size=40] 自选水果 x 2[/font_size]。\n点击闪烁的水果图标，挑选想要的吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>除了无限供应的盲盒，其他商品出售后都会暂时缺货。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>目前有两种升级可选。\n不如先买“解锁商店刷新”？</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>有些升级项可以反复购买，等级和效果随之提升。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>商店会在</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFC00000"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[color=#BC3D37]每天 00:00 [/color]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>上架随机商品，同时重置3次手动刷新次数。</t>
+    <r>
+      <t>除了</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>水果任务</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">，有时也会接到[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>传信任务</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">“感谢！给你[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>交换券</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> x 1[/font_size]，有空的话去附近的商店看看吧。”</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>商店</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>开张，可以用</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>交换券</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>购物了。\n进去看看吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>其他商品有点贵。\n不如先买个</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>盲盒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>碰碰运气？</t>
     </r>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -446,11 +879,10 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
       <t>升级券</t>
@@ -472,7 +904,26 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[font_size=40] 升级[/font_size]</t>
+      <t xml:space="preserve">[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>升级</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]</t>
     </r>
     <r>
       <rPr>
@@ -488,135 +939,158 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>获得了[font_size=40] 商店升级券 x 1[/font_size]。\n去商店升级格看看吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>现在请从商店获取[font_size=40][color=#94b757] 天平 [/color] x 1 [/font_size]吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>提升各类点数可以增加冒险成功率。\n不过需要四种点数共同作用，效果才会显著哦。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>四类点数道具会在对应的商店出售。\n目前没有商店能买到其他三类呢，先发放一些道具以作说明吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>冒险成功率提升了！\n道具准备越充分，就越能够避免冒险失败的情况。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>TUTORIAL_POINTS_7</t>
-  </si>
-  <si>
-    <t>TUTORIAL_POINTS_8</t>
-  </si>
-  <si>
-    <t>TUTORIAL_POINTS_9</t>
-  </si>
-  <si>
-    <r>
-      <t>如果</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[font_size=40] 失败 [/font_size]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>的话...就[color=#BC3D37] 一无所获 [/color]了呢。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>此外，游戏一共有[color=#BC3D37] 60 天[/color]的时间。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>花费更多时间在城里囤积道具的话，可用于出城冒险的时间则会相应减少。\n能够获得的[color=#BC3D37]  冒险得分 [/color]也会随天数降低。请注意。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>游戏的目标是获取更高的[color=#BC3D37]  冒险得分[/color]。\n因此, 在城里囤积道具的同时，努力留出更多时间用来冒险吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>You're ready to proceed.</t>
-  </si>
-  <si>
-    <t>Skip Tutorial</t>
-  </si>
-  <si>
-    <t>Welcome to the Tutorial.</t>
-  </si>
-  <si>
-    <t>Move your mouse along the tiles to plan a path,\nthen click the destination to confirm.</t>
-  </si>
-  <si>
-    <t>Are you sure to skip the tutorial?</t>
-  </si>
-  <si>
-    <t>Each move takes [color=#BC3D37]3 hours[/color]. Keep that in mind.</t>
-  </si>
-  <si>
-    <t>“Could you deliver a message to the Giraffe for me? Please!”</t>
-  </si>
-  <si>
-    <t>Other items are a bit pricey for now.\nHow about trying a Mystery Box instead?</t>
-  </si>
-  <si>
-    <t>Adventure success rate increased!\nThe more items you prepare, the less likely you are to fail.</t>
-  </si>
-  <si>
-    <t>Spending more time stocking up in the city means less time left for adventures.\nYour [color=#BC3D37]Adventure Score[/color] will also decrease as days pass. Keep that in mind.</t>
-  </si>
-  <si>
-    <t>The goal is to achieve a higher [color=#BC3D37]Adventure Score[/color].\nSo, stock up efficiently and leave more time for the adventure itself!</t>
-  </si>
-  <si>
-    <t>The game lasts [color=#BC3D37]60 days[/color] in total.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>准备妥当的话，就前往城门结束教程，正式开始游戏吧。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Just [font_size=40]Grapes x 1[/font_size] left to complete the quest.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Try stopping on that strange tile over there.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“Thanks for the fruit! Here are [font_size=40]Exchange Coupons x 2[/font_size].\nYou can use them at the shop.”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“I need [font_size=40]Apple x 1[/font_size] and [font_size=40]Grapes x1[/font_size], please!”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Another [font_size=40]Quest[/font_size]? Go pay them a visit.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>You got [font_size=40]Fruit of Your Choice x 2[/font_size]!\nClick the glowing fruit icons to pick the ones you want.</t>
+    <r>
+      <t>除了无限供应的</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>盲盒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>，其他商品出售后都会暂时缺货。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">获得了[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>商店升级券 x 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]。\n去</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>商店升级格</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>看看吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>目前有两种升级可选。\n不如先买“</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>解锁商店刷新</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>”？</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">现在请从商店购买[font_size=40][color=#94b757] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>天平</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [/color] x 1 [/font_size]吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">另一位似乎也有[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>任务</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]？拜访看看吧。</t>
+    </r>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
@@ -634,11 +1108,10 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
       <t>升级券</t>
@@ -661,80 +1134,160 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>呢。\n先努力获取[font_size=40] 交换券[/font_size]，再去升级格购买吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">There are currently two upgrades available.\nHow about buying “Shop Manual Refresh” first?  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>[font_size=40][color=#94b757]天平[/color][/font_size] 可以提供[font_size=40] 3 商店点数[/font_size]。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Raising different types of points increases adventure success rate.\nBut only when all four types work together will the effect be significant.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>[font_size=40][color=#94b757]Balance[/color][/font_size] provides [font_size=40]3 Shop Pts[/font_size].</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>It's time to get prepared in the city for the upcoming adventure.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>You got [font_size=40]Apple x 1[/font_size]!\nNot sure what it's for yet...</t>
+      <t xml:space="preserve">呢。\n先努力获取[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>交换券</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]，再去</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>商店</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>购买吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>[font_size=40][color=#94b757]</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>天平</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/color][/font_size] 可以提供[font_size=40] 3 商店点数[/font_size]。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Sometimes you'll also receive [font_size=40]</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>message delivery Quests</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[/font_size], \nnot just </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>fruit Quests</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
     <t>“Thanks for the message! Here's [font_size=40]Exchange Coupon x 1[/font_size].\nCheck out the nearby shop when you can.”</t>
-  </si>
-  <si>
-    <t>The four types of items are sold at their respective shops.\nThey're not available yet, so let's give you some for demonstration.</t>
-  </si>
-  <si>
-    <t>If you [font_size=40]fail[/font_size]... you'll return [color=#BC3D37]empty-handed[/color].</t>
-  </si>
-  <si>
-    <t>Unlike [font_size=40]Accepting Quests[/font_size],\n[font_size=40]Completing Quests[/font_size] doesn't require stopping on the tile. \nPassing through will automatically deliver them.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Sometimes you'll also receive [font_size=40]message delivery Quests[/font_size], \nnot just fruit ones.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">At the [font_size=40]Upgrade Tile[/font_size], \nyou can use [font_size=40]Upgrade Coupons[/font_size] to purchase various [font_size=40]Upgrades[/font_size].  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">You don't have any [font_size=40]Upgrade Coupons[/font_size] yet.\nFirst, try to earn some [font_size=40]Exchange Coupons[/font_size], \nthen head to the tile to buy upgrades.  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>You obtained [font_size=40]Shop Upgrade Coupon x 1[/font_size].\nGo check the shop upgrade tile.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Every day at [color=#BC3D37]00:00[/color], \nthe shop restocks with random items and also resets your 3 manual refresh uses.  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Aside from the unlimited Mystery Boxes, \nall other items will be temporarily out of stock after being sold.  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Some upgrades can be purchased multiple times, \nincreasing both their level and effectiveness.  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Now, please buy [font_size=40][color=#94b757]Balance[/color] x 1[/font_size] from the shop.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>When you're ready, \nhead to the city gate to end the tutorial and begin your adventure.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">You don't have any [font_size=40]Upgrade Coupons[/font_size] yet.\nGather some [font_size=40]Exchange Coupons[/font_size] first, \nthen visit the shop to buy one.  </t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Aside from the unlimited </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mystery Boxes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, \nall o ther items will be temporarily out of stock after being sold.  </t>
+    </r>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1387,7 +1940,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1403,50 +1956,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="20% - 着色 1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - 着色 2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - 着色 3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - 着色 4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - 着色 5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - 着色 6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - 着色 1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - 着色 2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - 着色 3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - 着色 4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - 着色 5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - 着色 6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - 着色 1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - 着色 2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - 着色 3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - 着色 4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - 着色 5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - 着色 6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="标题" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="标题 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="标题 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="标题 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="标题 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="差" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="好" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="汇总" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="计算" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="检查单元格" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="解释性文本" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="警告文本" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="链接单元格" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="适中" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="输出" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="输入" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="着色 1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="着色 2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="着色 3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="着色 4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="着色 5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="着色 6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="注释" xfId="15" builtinId="10" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1462,9 +2018,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1502,7 +2058,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1608,7 +2164,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1750,7 +2306,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1759,11 +2315,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D1D195-E5E8-4810-8E47-E25327235024}">
   <dimension ref="A1:C58"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="23.125" customWidth="1"/>
-    <col min="2" max="2" width="94.375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="83.625" customWidth="1"/>
+    <col min="1" max="1" width="23.08203125" customWidth="1"/>
+    <col min="2" max="2" width="94.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="83.58203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1793,7 +2349,7 @@
         <v>25</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>33</v>
@@ -1801,24 +2357,24 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1826,21 +2382,21 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1851,7 +2407,7 @@
         <v>36</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1859,10 +2415,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1870,10 +2426,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1887,10 +2443,10 @@
         <v>7</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1898,10 +2454,10 @@
         <v>8</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>60</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1925,10 +2481,10 @@
         <v>9</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>40</v>
+        <v>108</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>61</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1936,10 +2492,10 @@
         <v>10</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1947,10 +2503,10 @@
         <v>11</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>62</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1972,18 +2528,18 @@
         <v>38</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="28.5">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="28">
       <c r="A23" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1991,10 +2547,10 @@
         <v>15</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>66</v>
+        <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -2014,10 +2570,10 @@
         <v>16</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>67</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -2025,10 +2581,10 @@
         <v>17</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -2036,21 +2592,21 @@
         <v>18</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="28.5">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="28">
       <c r="A31" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>70</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2066,10 +2622,10 @@
         <v>19</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>71</v>
+        <v>41</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -2077,10 +2633,10 @@
         <v>20</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>72</v>
+        <v>117</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -2088,10 +2644,10 @@
         <v>21</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -2102,26 +2658,26 @@
       <c r="A38" s="4"/>
       <c r="C38" s="4"/>
     </row>
-    <row r="39" spans="1:3" ht="28.5">
+    <row r="39" spans="1:3" ht="28">
       <c r="A39" s="4" t="s">
         <v>22</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="28.5">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="28">
       <c r="A40" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -2129,21 +2685,21 @@
         <v>27</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="28.5">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="28">
       <c r="A42" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -2151,10 +2707,10 @@
         <v>29</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
@@ -2162,10 +2718,10 @@
         <v>30</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>75</v>
+        <v>121</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
@@ -2173,10 +2729,10 @@
         <v>31</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="14.25" customHeight="1">
@@ -2193,101 +2749,101 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>80</v>
+        <v>122</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="28">
+      <c r="A51" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="28.5">
-      <c r="A51" s="4" t="s">
+      <c r="B51" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="28">
+      <c r="A52" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="28.5">
-      <c r="A52" s="4" t="s">
-        <v>46</v>
-      </c>
       <c r="B52" s="4" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="28">
+      <c r="A56" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="28">
+      <c r="A57" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" ht="28.5">
-      <c r="A56" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="28.5">
-      <c r="A57" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>101</v>
-      </c>
       <c r="C57" s="4" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -2295,10 +2851,10 @@
         <v>32</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: Now tutorial will lock input
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Tutorial_String_Data.xlsx
+++ b/Assets/Internationalization/Tutorial_String_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\city_of_circling\city_of_circling\Assets\Internationalization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A71328-EA98-4F2C-915D-A068F8CCCD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA914C43-ABB2-4E15-A654-59807F139A71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="1250" windowWidth="38620" windowHeight="21100" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
+    <workbookView xWindow="25490" yWindow="-7310" windowWidth="21820" windowHeight="37900" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
   <sheets>
     <sheet name="String_Data" sheetId="1" r:id="rId1"/>
@@ -52,9 +52,6 @@
     <t>TUTORIAL_NPC_1</t>
   </si>
   <si>
-    <t>TUTORIAL_NPC_2</t>
-  </si>
-  <si>
     <t>TUTORIAL_NPC_3</t>
   </si>
   <si>
@@ -497,9 +494,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">“我需要[font_size=40] </t>
-    </r>
-    <r>
       <rPr>
         <b/>
         <sz val="11"/>
@@ -507,7 +501,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>苹果 x 1</t>
+      <t>商店</t>
     </r>
     <r>
       <rPr>
@@ -518,7 +512,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">[/font_size] 和[font_size=40] </t>
+      <t>开张，可以用</t>
     </r>
     <r>
       <rPr>
@@ -528,7 +522,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>葡萄 x 1</t>
+      <t>交换券</t>
     </r>
     <r>
       <rPr>
@@ -539,13 +533,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size]，拜托了！”</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">还差[font_size=40] </t>
+      <t>购物了。\n进去看看吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>其他商品有点贵。\n不如先买个</t>
     </r>
     <r>
       <rPr>
@@ -555,7 +549,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>葡萄 x 1</t>
+      <t>盲盒</t>
     </r>
     <r>
       <rPr>
@@ -566,13 +560,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size] 就能完成任务。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">获得了[font_size=40] </t>
+      <t>碰碰运气？</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>在</t>
     </r>
     <r>
       <rPr>
@@ -582,7 +576,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>苹果 x 1</t>
+      <t>[font_size=40] 升级格 [/font_size]</t>
     </r>
     <r>
       <rPr>
@@ -593,13 +587,16 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size]。\n虽然不知道能用来做什么...</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">“感谢你的水果！送你[font_size=40] </t>
+      <t>可以用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[font_size=40] </t>
     </r>
     <r>
       <rPr>
@@ -609,7 +606,45 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>交换券 x 2</t>
+      <t>升级券</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [/font_size]购买各种</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>升级</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[/font_size]</t>
     </r>
     <r>
       <rPr>
@@ -620,13 +655,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size]，可以用来在商店购物哦。”</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">不同于[font_size=40] </t>
+      <t>。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>除了无限供应的</t>
     </r>
     <r>
       <rPr>
@@ -636,7 +671,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>接受任务</t>
+      <t>盲盒</t>
     </r>
     <r>
       <rPr>
@@ -647,11 +682,26 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size]，\n</t>
+      <t>，其他商品出售后都会暂时缺货。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">获得了[font_size=40] </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>商店升级券 x 1</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="等线"/>
@@ -659,7 +709,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[font_size=40]完成</t>
+      <t>[/font_size]。\n去</t>
     </r>
     <r>
       <rPr>
@@ -669,11 +719,10 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>任务</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
+      <t>商店升级格</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="等线"/>
@@ -681,7 +730,23 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> [/font_size]</t>
+      <t>看看吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>目前有两种升级可选。\n不如先买“</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>解锁商店刷新</t>
     </r>
     <r>
       <rPr>
@@ -692,13 +757,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>时不需要停留在格子上，路过就会自动交付。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>除了</t>
+      <t>”？</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">现在请从商店购买[font_size=40][color=#94b757] </t>
     </r>
     <r>
       <rPr>
@@ -708,7 +773,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>水果任务</t>
+      <t>天平</t>
     </r>
     <r>
       <rPr>
@@ -719,17 +784,22 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">，有时也会接到[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>传信任务</t>
+      <t xml:space="preserve"> [/color] x 1 [/font_size]吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">另一位似乎也有[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>任务</t>
     </r>
     <r>
       <rPr>
@@ -740,13 +810,22 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size]。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">“感谢！给你[font_size=40] </t>
+      <t>[/font_size]？拜访看看吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>现在还没有</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[font_size=40] </t>
     </r>
     <r>
       <rPr>
@@ -756,7 +835,16 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>交换券</t>
+      <t>升级券</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [/font_size]</t>
     </r>
     <r>
       <rPr>
@@ -767,11 +855,8 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> x 1[/font_size]，有空的话去附近的商店看看吧。”</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
+      <t xml:space="preserve">呢。\n先努力获取[font_size=40] </t>
+    </r>
     <r>
       <rPr>
         <b/>
@@ -780,7 +865,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>商店</t>
+      <t>交换券</t>
     </r>
     <r>
       <rPr>
@@ -791,7 +876,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>开张，可以用</t>
+      <t>[/font_size]，再去</t>
     </r>
     <r>
       <rPr>
@@ -801,7 +886,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>交换券</t>
+      <t>商店</t>
     </r>
     <r>
       <rPr>
@@ -812,13 +897,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>购物了。\n进去看看吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>其他商品有点贵。\n不如先买个</t>
+      <t>购买吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>[font_size=40][color=#94b757]</t>
     </r>
     <r>
       <rPr>
@@ -828,7 +913,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>盲盒</t>
+      <t>天平</t>
     </r>
     <r>
       <rPr>
@@ -839,13 +924,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>碰碰运气？</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>在</t>
+      <t>[/color][/font_size] 可以提供[font_size=40] 3 商店点数[/font_size]。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Sometimes you'll also receive [font_size=40]</t>
     </r>
     <r>
       <rPr>
@@ -855,7 +940,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[font_size=40] 升级格 [/font_size]</t>
+      <t>message delivery Quests</t>
     </r>
     <r>
       <rPr>
@@ -866,16 +951,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>可以用</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[font_size=40] </t>
+      <t xml:space="preserve">[/font_size], \nnot just </t>
     </r>
     <r>
       <rPr>
@@ -885,45 +961,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>升级券</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> [/font_size]购买各种</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>升级</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[/font_size]</t>
+      <t>fruit Quests</t>
     </r>
     <r>
       <rPr>
@@ -934,13 +972,21 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>除了无限供应的</t>
+      <t>.</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“Thanks for the message! Here's [font_size=40]Exchange Coupon x 1[/font_size].\nCheck out the nearby shop when you can.”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">You don't have any [font_size=40]Upgrade Coupons[/font_size] yet.\nGather some [font_size=40]Exchange Coupons[/font_size] first, \nthen visit the shop to buy one.  </t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Aside from the unlimited </t>
     </r>
     <r>
       <rPr>
@@ -950,7 +996,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>盲盒</t>
+      <t>Mystery Boxes</t>
     </r>
     <r>
       <rPr>
@@ -961,23 +1007,30 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>，其他商品出售后都会暂时缺货。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">获得了[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>商店升级券 x 1</t>
+      <t xml:space="preserve">, \nall o ther items will be temporarily out of stock after being sold.  </t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>获得了[img={"height":"60"}]res://Assets/Sprites/Icon/1x/apple.png[/img][font_size=40]苹果 x 1[/font_size]。\n虽然不知道能用来做什么…</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“我需要[img={"height":"60"}]res://Assets/Sprites/Icon/1x/apple.png[/img][font_size=40]苹果 x 1[/font_size] 和[img={"height":"60"}]res://Assets/Sprites/Icon/1x/grape.png[/img][font_size=40]葡萄 x 1[/font_size]，拜托了！”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>还差</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[img={"height":"60"}]res://Assets/Sprites/Icon/1x/grape.png[/img]</t>
     </r>
     <r>
       <rPr>
@@ -988,7 +1041,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size]。\n去</t>
+      <t>[font_size=40]</t>
     </r>
     <r>
       <rPr>
@@ -998,7 +1051,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>商店升级格</t>
+      <t>葡萄 x 1</t>
     </r>
     <r>
       <rPr>
@@ -1009,13 +1062,29 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>看看吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>目前有两种升级可选。\n不如先买“</t>
+      <t>[/font_size] 就能完成任务。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>不同于 [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_new.png[/img] [font_size=40]接受任务[/font_size]，\n [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_complete.png[/img] [font_size=40]完成任务 [/font_size]时不需要停留在格子上，路过就会自动交付。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>TUTORIAL_NPC_2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“感谢你的水果！送你 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]交换券 x 2[/font_size]，可以用来在商店购物哦。”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>除了 [img={"height":"40"}]res://Assets/Sprites/Icon/1x/Quest_fruit.png[/img] [font_size=40]水果任务[/font_size]，有时也会接到 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/Quest_delivery.png[/img] [font_size=40]传信任务[/font_size]。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>“感谢！给你 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]</t>
     </r>
     <r>
       <rPr>
@@ -1025,7 +1094,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>解锁商店刷新</t>
+      <t>交换券</t>
     </r>
     <r>
       <rPr>
@@ -1036,257 +1105,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>”？</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">现在请从商店购买[font_size=40][color=#94b757] </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>天平</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> [/color] x 1 [/font_size]吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">另一位似乎也有[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>任务</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[/font_size]？拜访看看吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>现在还没有</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>升级券</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> [/font_size]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">呢。\n先努力获取[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>交换券</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[/font_size]，再去</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>商店</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>购买吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>[font_size=40][color=#94b757]</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>天平</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[/color][/font_size] 可以提供[font_size=40] 3 商店点数[/font_size]。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>Sometimes you'll also receive [font_size=40]</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>message delivery Quests</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[/font_size], \nnot just </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>fruit Quests</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“Thanks for the message! Here's [font_size=40]Exchange Coupon x 1[/font_size].\nCheck out the nearby shop when you can.”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">You don't have any [font_size=40]Upgrade Coupons[/font_size] yet.\nGather some [font_size=40]Exchange Coupons[/font_size] first, \nthen visit the shop to buy one.  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Aside from the unlimited </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Mystery Boxes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, \nall o ther items will be temporarily out of stock after being sold.  </t>
+      <t xml:space="preserve"> x 1[/font_size]，有空的话去附近的商店看看吧。”</t>
     </r>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -1961,48 +1780,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - 着色 1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="标题" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="标题 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="标题 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="标题 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="标题 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="差" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="好" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="汇总" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="计算" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="检查单元格" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="解释性文本" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="警告文本" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="链接单元格" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="适中" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="输出" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="输入" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="着色 1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="着色 2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="着色 3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="着色 4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="着色 5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="着色 6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="注释" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2018,9 +1837,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2058,7 +1877,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2164,7 +1983,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2306,7 +2125,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2315,11 +2134,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D1D195-E5E8-4810-8E47-E25327235024}">
   <dimension ref="A1:C58"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="23.08203125" customWidth="1"/>
-    <col min="2" max="2" width="94.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="83.58203125" customWidth="1"/>
+    <col min="1" max="1" width="23.125" customWidth="1"/>
+    <col min="2" max="2" width="94.375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="83.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2335,46 +2154,46 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2382,21 +2201,21 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -2404,10 +2223,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2415,10 +2234,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -2426,15 +2245,15 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" s="4"/>
     </row>
@@ -2443,21 +2262,21 @@
         <v>7</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="28.5">
       <c r="A13" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -2481,76 +2300,76 @@
         <v>9</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="42.75">
       <c r="A19" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="28.5">
+      <c r="A20" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="B20" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="42.75">
+      <c r="A23" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="28">
-      <c r="A23" s="4" t="s">
+      <c r="B23" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="28.5">
+      <c r="A24" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="4" t="s">
-        <v>15</v>
-      </c>
       <c r="B24" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -2567,46 +2386,46 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="42.75">
+      <c r="A30" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="4" t="s">
-        <v>18</v>
-      </c>
       <c r="B30" s="4" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="28">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="28.5">
       <c r="A31" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2619,35 +2438,35 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -2658,81 +2477,81 @@
       <c r="A38" s="4"/>
       <c r="C38" s="4"/>
     </row>
-    <row r="39" spans="1:3" ht="28">
+    <row r="39" spans="1:3" ht="28.5">
       <c r="A39" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="28.5">
+      <c r="A40" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="28">
-      <c r="A40" s="4" t="s">
-        <v>23</v>
-      </c>
       <c r="B40" s="4" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="28.5">
+      <c r="A42" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="28">
-      <c r="A42" s="4" t="s">
-        <v>28</v>
-      </c>
       <c r="B42" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
       <c r="A44" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
       <c r="A45" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="14.25" customHeight="1">
@@ -2749,112 +2568,112 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="28.5">
+      <c r="A51" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="28">
-      <c r="A51" s="4" t="s">
+      <c r="B51" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="28.5">
+      <c r="A52" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C51" s="4" t="s">
+      <c r="B52" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C52" s="4" t="s">
         <v>64</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="28">
-      <c r="A52" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="28.5">
+      <c r="A56" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C55" s="4" t="s">
+      <c r="B56" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C56" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="28">
-      <c r="A56" s="4" t="s">
+    <row r="57" spans="1:3" ht="28.5">
+      <c r="A57" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B57" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C57" s="4" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="28">
-      <c r="A57" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: Icon added to tutorial text
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Tutorial_String_Data.xlsx
+++ b/Assets/Internationalization/Tutorial_String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA914C43-ABB2-4E15-A654-59807F139A71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E53A13-337C-412A-AAB8-8A3BAF8092B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-7310" windowWidth="21820" windowHeight="37900" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
@@ -146,9 +146,6 @@
     <t>TUTORIAL_NPC_11</t>
   </si>
   <si>
-    <t>The shop is open! You can buy things with Exchange Coupons.\nTake a look.</t>
-  </si>
-  <si>
     <t>TUTORIAL_POINTS_1</t>
   </si>
   <si>
@@ -388,9 +385,6 @@
     <t>“Could you deliver a message to the Giraffe for me? Please!”</t>
   </si>
   <si>
-    <t>Other items are a bit pricey for now.\nHow about trying a Mystery Box instead?</t>
-  </si>
-  <si>
     <t>Adventure success rate increased!\nThe more items you prepare, the less likely you are to fail.</t>
   </si>
   <si>
@@ -400,108 +394,31 @@
     <t>The goal is to achieve a higher [color=#BC3D37]Adventure Score[/color].\nSo, stock up efficiently and leave more time for the adventure itself!</t>
   </si>
   <si>
-    <t>The game lasts [color=#BC3D37]60 days[/color] in total.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>准备妥当的话，就前往城门结束教程，正式开始游戏吧。</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>Just [font_size=40]Grapes x 1[/font_size] left to complete the quest.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Try stopping on that strange tile over there.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“Thanks for the fruit! Here are [font_size=40]Exchange Coupons x 2[/font_size].\nYou can use them at the shop.”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“I need [font_size=40]Apple x 1[/font_size] and [font_size=40]Grapes x1[/font_size], please!”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Another [font_size=40]Quest[/font_size]? Go pay them a visit.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>You got [font_size=40]Fruit of Your Choice x 2[/font_size]!\nClick the glowing fruit icons to pick the ones you want.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">There are currently two upgrades available.\nHow about buying “Shop Manual Refresh” first?  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Raising different types of points increases adventure success rate.\nBut only when all four types work together will the effect be significant.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>[font_size=40][color=#94b757]Balance[/color][/font_size] provides [font_size=40]3 Shop Pts[/font_size].</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>It's time to get prepared in the city for the upcoming adventure.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>You got [font_size=40]Apple x 1[/font_size]!\nNot sure what it's for yet...</t>
-  </si>
-  <si>
     <t>The four types of items are sold at their respective shops.\nThey're not available yet, so let's give you some for demonstration.</t>
   </si>
   <si>
     <t>If you [font_size=40]fail[/font_size]... you'll return [color=#BC3D37]empty-handed[/color].</t>
   </si>
   <si>
-    <t>Unlike [font_size=40]Accepting Quests[/font_size],\n[font_size=40]Completing Quests[/font_size] doesn't require stopping on the tile. \nPassing through will automatically deliver them.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">At the [font_size=40]Upgrade Tile[/font_size], \nyou can use [font_size=40]Upgrade Coupons[/font_size] to purchase various [font_size=40]Upgrades[/font_size].  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>You obtained [font_size=40]Shop Upgrade Coupon x 1[/font_size].\nGo check the shop upgrade tile.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Every day at [color=#BC3D37]00:00[/color], \nthe shop restocks with random items and also resets your 3 manual refresh uses.  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Some upgrades can be purchased multiple times, \nincreasing both their level and effectiveness.  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Now, please buy [font_size=40][color=#94b757]Balance[/color] x 1[/font_size] from the shop.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>When you're ready, \nhead to the city gate to end the tutorial and begin your adventure.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>似乎有人正在发布任务。\n去拜访看看吧。</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>Seems like someone's posting a quest.\nGo pay them a visit.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>商店</t>
+    <r>
+      <t xml:space="preserve">另一位似乎也有[font_size=40] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>任务</t>
     </r>
     <r>
       <rPr>
@@ -512,17 +429,30 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>开张，可以用</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>交换券</t>
+      <t>[/font_size]？拜访看看吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>获得了[img={"height":"60"}]res://Assets/Sprites/Icon/1x/apple.png[/img][font_size=40]苹果 x 1[/font_size]。\n虽然不知道能用来做什么…</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“我需要[img={"height":"60"}]res://Assets/Sprites/Icon/1x/apple.png[/img][font_size=40]苹果 x 1[/font_size] 和[img={"height":"60"}]res://Assets/Sprites/Icon/1x/grape.png[/img][font_size=40]葡萄 x 1[/font_size]，拜托了！”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>还差</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[img={"height":"60"}]res://Assets/Sprites/Icon/1x/grape.png[/img]</t>
     </r>
     <r>
       <rPr>
@@ -533,13 +463,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>购物了。\n进去看看吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>其他商品有点贵。\n不如先买个</t>
+      <t>[font_size=40]</t>
     </r>
     <r>
       <rPr>
@@ -549,7 +473,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>盲盒</t>
+      <t>葡萄 x 1</t>
     </r>
     <r>
       <rPr>
@@ -560,13 +484,29 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>碰碰运气？</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>在</t>
+      <t>[/font_size] 就能完成任务。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>不同于 [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_new.png[/img] [font_size=40]接受任务[/font_size]，\n [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_complete.png[/img] [font_size=40]完成任务 [/font_size]时不需要停留在格子上，路过就会自动交付。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>TUTORIAL_NPC_2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“感谢你的水果！送你 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]交换券 x 2[/font_size]，可以用来在商店购物哦。”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>除了 [img={"height":"40"}]res://Assets/Sprites/Icon/1x/Quest_fruit.png[/img] [font_size=40]水果任务[/font_size]，有时也会接到 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/Quest_delivery.png[/img] [font_size=40]传信任务[/font_size]。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>“感谢！给你 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]</t>
     </r>
     <r>
       <rPr>
@@ -576,7 +516,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[font_size=40] 升级格 [/font_size]</t>
+      <t>交换券</t>
     </r>
     <r>
       <rPr>
@@ -587,16 +527,33 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>可以用</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[font_size=40] </t>
+      <t xml:space="preserve"> x 1[/font_size]，有空的话去附近的商店看看吧。”</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>[img={"height":"45"}]res://Assets/Sprites/Icon/1x/trade_shop.png[/img] [font_size=40]商店[/font_size] 开张，可以用 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]交换券 [/font_size]购物了。\n进去看看吧。</t>
+  </si>
+  <si>
+    <t>其他商品有点贵。\n不如先买个[img={"height":"60"}]res://Assets/Sprites/Icon/1x/mystery_box.png[/img][font_size=40]盲盒[/font_size] 碰碰运气？</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>在 [img={"height":"45"}]res://Assets/Sprites/Grid/1x/shop_upgrade.png[/img][font_size=40] 升级格 [/font_size]可以用[img={"height":"60"}]res://Assets/Sprites/Icon/1x/trade upgrade coupon.png[/img][font_size=40]升级券 [/font_size]购买各种[font_size=40] 升级[/font_size]。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>现在还没有</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[img={"height":"60"}]res://Assets/Sprites/Icon/1x/trade upgrade coupon.png[/img][font_size=40]</t>
     </r>
     <r>
       <rPr>
@@ -615,36 +572,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> [/font_size]购买各种</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>升级</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[/font_size]</t>
+      <t xml:space="preserve"> [/font_size]</t>
     </r>
     <r>
       <rPr>
@@ -655,13 +583,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>除了无限供应的</t>
+      <t>呢。\n先努力获取 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]</t>
     </r>
     <r>
       <rPr>
@@ -671,7 +593,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>盲盒</t>
+      <t>交换券</t>
     </r>
     <r>
       <rPr>
@@ -682,13 +604,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>，其他商品出售后都会暂时缺货。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">获得了[font_size=40] </t>
+      <t>[/font_size]，再去</t>
     </r>
     <r>
       <rPr>
@@ -698,7 +614,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>商店升级券 x 1</t>
+      <t>商店</t>
     </r>
     <r>
       <rPr>
@@ -709,7 +625,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size]。\n去</t>
+      <t>购买吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>除了无限供应的[img={"height":"60"}]res://Assets/Sprites/Icon/1x/mystery_box.png[/img]</t>
     </r>
     <r>
       <rPr>
@@ -719,7 +641,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>商店升级格</t>
+      <t>盲盒</t>
     </r>
     <r>
       <rPr>
@@ -730,23 +652,22 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>看看吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>目前有两种升级可选。\n不如先买“</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>解锁商店刷新</t>
+      <t>，其他商品出售后都会暂时缺货。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>获得了</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[img={"height":"60"}]res://Assets/Sprites/Icon/1x/trade upgrade coupon.png[/img]</t>
     </r>
     <r>
       <rPr>
@@ -757,13 +678,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>”？</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">现在请从商店购买[font_size=40][color=#94b757] </t>
+      <t>[font_size=40]</t>
     </r>
     <r>
       <rPr>
@@ -773,7 +688,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>天平</t>
+      <t>商店升级券 x 1</t>
     </r>
     <r>
       <rPr>
@@ -784,22 +699,17 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> [/color] x 1 [/font_size]吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">另一位似乎也有[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>任务</t>
+      <t xml:space="preserve">[/font_size]。\n去 [img={"height":"45"}]res://Assets/Sprites/Grid/1x/shop_upgrade.png[/img] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>商店升级格</t>
     </r>
     <r>
       <rPr>
@@ -810,22 +720,21 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[/font_size]？拜访看看吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>现在还没有</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[font_size=40] </t>
+      <t>看看吧。</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>目前有两种升级可选。\n不如先买[img={"height":"60"}]res://Assets/Sprites/Icon/1x/shop_manual_refresh.png[/img]“解锁商店刷新”？</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>现在请再次前往商店购买 [img={"height":"60"}]res://Assets/Sprites/Icon/1x/balance.png[/img][font_size=40][color=#94b757] 天平 [/color] x 1 [/font_size]吧。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>[img={"height":"60"}]res://Assets/Sprites/Icon/1x/balance.png[/img] [font_size=40][color=#94b757]</t>
     </r>
     <r>
       <rPr>
@@ -835,16 +744,7 @@
         <rFont val="等线"/>
         <scheme val="minor"/>
       </rPr>
-      <t>升级券</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> [/font_size]</t>
+      <t>天平</t>
     </r>
     <r>
       <rPr>
@@ -855,258 +755,97 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">呢。\n先努力获取[font_size=40] </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>交换券</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[/font_size]，再去</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>商店</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>购买吧。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>[font_size=40][color=#94b757]</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>天平</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>[/color][/font_size] 可以提供[font_size=40] 3 商店点数[/font_size]。</t>
     </r>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t>Sometimes you'll also receive [font_size=40]</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>message delivery Quests</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[/font_size], \nnot just </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>fruit Quests</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“Thanks for the message! Here's [font_size=40]Exchange Coupon x 1[/font_size].\nCheck out the nearby shop when you can.”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">You don't have any [font_size=40]Upgrade Coupons[/font_size] yet.\nGather some [font_size=40]Exchange Coupons[/font_size] first, \nthen visit the shop to buy one.  </t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Aside from the unlimited </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Mystery Boxes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, \nall o ther items will be temporarily out of stock after being sold.  </t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>获得了[img={"height":"60"}]res://Assets/Sprites/Icon/1x/apple.png[/img][font_size=40]苹果 x 1[/font_size]。\n虽然不知道能用来做什么…</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“我需要[img={"height":"60"}]res://Assets/Sprites/Icon/1x/apple.png[/img][font_size=40]苹果 x 1[/font_size] 和[img={"height":"60"}]res://Assets/Sprites/Icon/1x/grape.png[/img][font_size=40]葡萄 x 1[/font_size]，拜托了！”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>还差</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[img={"height":"60"}]res://Assets/Sprites/Icon/1x/grape.png[/img]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[font_size=40]</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>葡萄 x 1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[/font_size] 就能完成任务。</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>不同于 [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_new.png[/img] [font_size=40]接受任务[/font_size]，\n [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_complete.png[/img] [font_size=40]完成任务 [/font_size]时不需要停留在格子上，路过就会自动交付。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>TUTORIAL_NPC_2</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>“感谢你的水果！送你 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]交换券 x 2[/font_size]，可以用来在商店购物哦。”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>除了 [img={"height":"40"}]res://Assets/Sprites/Icon/1x/Quest_fruit.png[/img] [font_size=40]水果任务[/font_size]，有时也会接到 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/Quest_delivery.png[/img] [font_size=40]传信任务[/font_size]。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>“感谢！给你 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>交换券</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> x 1[/font_size]，有空的话去附近的商店看看吧。”</t>
-    </r>
+    <t>It's time to get prepared in the city for the upcoming adventure.</t>
+  </si>
+  <si>
+    <t>Try stopping on that strange tile over there.</t>
+  </si>
+  <si>
+    <t>You got [img={"height":"60"}]res://Assets/Sprites/Icon/1x/apple.png[/img][font_size=40]Apple x 1[/font_size]!\nNot sure what it's for yet...</t>
+  </si>
+  <si>
+    <t>Seems like someone's posting a quest.\nGo pay them a visit.</t>
+  </si>
+  <si>
+    <t>“I need [img={"height":"60"}]res://Assets/Sprites/Icon/1x/apple.png[/img][font_size=40]Apple x 1[/font_size] and [img={"height":"60"}]res://Assets/Sprites/Icon/1x/grape.png[/img][font_size=40]Grapes x 1[/font_size], please!”</t>
+  </si>
+  <si>
+    <t>Just [img={"height":"60"}]res://Assets/Sprites/Icon/1x/grape.png[/img][font_size=40]Grapes x 1[/font_size] left to complete the quest.</t>
+  </si>
+  <si>
+    <t>You got [font_size=40]Fruit of Your Choice x 2[/font_size]!\nClick the glowing fruit icons to pick the ones you want.</t>
+  </si>
+  <si>
+    <t>Aside from the unlimited [img={"height":"60"}]res://Assets/Sprites/Icon/1x/mystery_box.png[/img][font_size=40]Mystery Boxes[/font_size],\nall other items will be temporarily out of stock after being sold.</t>
+  </si>
+  <si>
+    <t>Every day at [color=#BC3D37]00:00[/color],\nthe shop restocks with random items and also resets your 3 manual refresh uses.</t>
+  </si>
+  <si>
+    <t>You obtained [img={"height":"60"}]res://Assets/Sprites/Icon/1x/trade upgrade coupon.png[/img][font_size=40]Shop Upgrade Coupon x 1[/font_size].\nGo check the shop upgrade tile.</t>
+  </si>
+  <si>
+    <t>Some upgrades can be purchased multiple times,\nincreasing both their level and effectiveness.</t>
+  </si>
+  <si>
+    <t>[img={"height":"60"}]res://Assets/Sprites/Icon/1x/balance.png[/img][font_size=40][color=#94b757]Balance[/color][/font_size] provides [font_size=40]3 Shop Pts[/font_size].</t>
+  </si>
+  <si>
+    <t>Raising different types of points increases adventure success rate.\nBut only when all four types work together will the effect be significant.</t>
+  </si>
+  <si>
+    <t>The game lasts [color=#BC3D37]60 days[/color] in total.</t>
+  </si>
+  <si>
+    <t>When you're ready,\nhead to the city gate to end the tutorial and begin your adventure.</t>
+  </si>
+  <si>
+    <t>Unlike [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_new.png[/img] [font_size=40]Accepting Quests[/font_size],\n[img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_complete.png[/img] [font_size=40]Completing Quests[/font_size] doesn't require stopping on the tile.\nPassing through will automatically deliver them.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“Thanks for the fruit! Here are [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]Exchange Coupons x 2[/font_size].\nYou can use them at the shop.”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Another [font_size=40]Quest[/font_size]? Go pay them a visit.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sometimes you'll also receive [img={"height":"40"}]res://Assets/Sprites/Icon/1x/Quest_fruit.png[/img] [font_size=40]Message Delivery Quests[/font_size],\nnot just [img={"height":"50"}]res://Assets/Sprites/Icon/1x/Quest_delivery.png[/img] [font_size=40]Fruit Quests[/font_size].</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>“Thanks for the message! Here's [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]Exchange Coupon x 1[/font_size].\nCheck out the nearby shop when you can.”</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Other items are a bit pricey.\nHow about trying a [img={"height":"60"}]res://Assets/Sprites/Icon/1x/mystery_box.png[/img][font_size=40]Mystery Box[/font_size] instead?</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>At the [img={"height":"45"}]res://Assets/Sprites/Grid/1x/shop_upgrade.png[/img] [font_size=40]Upgrade Tile[/font_size],\nyou can use [img={"height":"60"}]res://Assets/Sprites/Icon/1x/trade upgrade coupon.png[/img][font_size=40]Upgrade Coupons[/font_size] to purchase various [font_size=40]Upgrades[/font_size].</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>You don't have any [img={"height":"60"}]res://Assets/Sprites/Icon/1x/trade upgrade coupon.png[/img][font_size=40]Upgrade Coupons[/font_size] yet.\nGather some [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]Exchange Coupons[/font_size] first,\nthen visit the shop to buy one.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>There are currently two upgrades available.\nHow about buying [img={"height":"60"}]res://Assets/Sprites/Icon/1x/shop_manual_refresh.png[/img][font_size=40]Shop Manual Refresh[/font_size] first?</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Now, please buy [img={"height":"60"}]res://Assets/Sprites/Icon/1x/balance.png[/img][font_size=40][color=#94b757]Balance[/color] x 1[/font_size] from the shop.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>[img={"height":"45"}]res://Assets/Sprites/Icon/1x/trade_shop.png[/img] [font_size=40]The shop[/font_size] is open!\nYou can buy things with [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]Exchange Coupons[/font_size].\nTake a look.</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -2137,18 +1876,18 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.125" customWidth="1"/>
-    <col min="2" max="2" width="94.375" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="83.625" customWidth="1"/>
+    <col min="2" max="2" width="90.375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="83.625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2156,10 +1895,10 @@
       <c r="A2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2167,88 +1906,88 @@
       <c r="A3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>75</v>
+      <c r="B6" s="1" t="s">
+        <v>74</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>95</v>
+        <v>50</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>104</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>76</v>
+      <c r="B9" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>78</v>
+      <c r="B10" s="1" t="s">
+        <v>77</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -2261,22 +2000,22 @@
       <c r="A12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>87</v>
+      <c r="B12" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="28.5">
       <c r="A13" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>96</v>
+      <c r="B13" s="1" t="s">
+        <v>106</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>122</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -2299,33 +2038,33 @@
       <c r="A18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="42.75">
       <c r="A19" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>108</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>123</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="28.5">
       <c r="A20" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>86</v>
+      <c r="B20" s="1" t="s">
+        <v>109</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>124</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -2347,29 +2086,29 @@
         <v>37</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="42.75">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="57">
       <c r="A23" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>99</v>
+      <c r="B23" s="1" t="s">
+        <v>119</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>125</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="28.5">
       <c r="A24" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>88</v>
+      <c r="B24" s="1" t="s">
+        <v>120</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -2388,44 +2127,44 @@
       <c r="A28" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>90</v>
+      <c r="B28" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>79</v>
+      <c r="B29" s="1" t="s">
+        <v>78</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="42.75">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="57">
       <c r="A30" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>118</v>
+      <c r="B30" s="1" t="s">
+        <v>122</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>128</v>
+        <v>93</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="28.5">
       <c r="A31" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>119</v>
+      <c r="B31" s="1" t="s">
+        <v>123</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2436,37 +2175,37 @@
       <c r="A33" s="4"/>
       <c r="C33" s="4"/>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" ht="42.75">
       <c r="A34" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>40</v>
+      <c r="B34" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="42.75">
       <c r="A35" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>80</v>
+      <c r="B35" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="28.5">
       <c r="A36" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -2477,70 +2216,70 @@
       <c r="A38" s="4"/>
       <c r="C38" s="4"/>
     </row>
-    <row r="39" spans="1:3" ht="28.5">
+    <row r="39" spans="1:3" ht="57">
       <c r="A39" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="28.5">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="57">
       <c r="A40" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>120</v>
+      <c r="B40" s="1" t="s">
+        <v>126</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="42.75">
       <c r="A41" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>121</v>
+      <c r="B41" s="1" t="s">
+        <v>111</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="28.5">
       <c r="A42" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B42" s="4" t="s">
-        <v>102</v>
+      <c r="B42" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="42.75">
       <c r="A43" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B43" s="4" t="s">
-        <v>101</v>
+      <c r="B43" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
       <c r="A44" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>92</v>
+      <c r="B44" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
@@ -2548,10 +2287,10 @@
         <v>30</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="14.25" customHeight="1">
@@ -2566,114 +2305,114 @@
       <c r="A48" s="4"/>
       <c r="C48" s="4"/>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" ht="42.75">
       <c r="A49" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="28.5">
+      <c r="A50" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>94</v>
+      <c r="B50" s="1" t="s">
+        <v>115</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="28.5">
       <c r="A51" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>93</v>
+        <v>42</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="28.5">
       <c r="A52" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>97</v>
+        <v>43</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>98</v>
+        <v>45</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>84</v>
+        <v>65</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="28.5">
       <c r="A56" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>82</v>
+        <v>66</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="28.5">
       <c r="A57" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>105</v>
+      <c r="B58" s="1" t="s">
+        <v>118</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FIXED: Icon Path Uppercase bug
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Tutorial_String_Data.xlsx
+++ b/Assets/Internationalization/Tutorial_String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E53A13-337C-412A-AAB8-8A3BAF8092B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BCBC676-A8AD-4C75-A94D-F0A2D9315FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-7310" windowWidth="21820" windowHeight="37900" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
@@ -489,19 +489,11 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>不同于 [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_new.png[/img] [font_size=40]接受任务[/font_size]，\n [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_complete.png[/img] [font_size=40]完成任务 [/font_size]时不需要停留在格子上，路过就会自动交付。</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>TUTORIAL_NPC_2</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
     <t>“感谢你的水果！送你 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]交换券 x 2[/font_size]，可以用来在商店购物哦。”</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>除了 [img={"height":"40"}]res://Assets/Sprites/Icon/1x/Quest_fruit.png[/img] [font_size=40]水果任务[/font_size]，有时也会接到 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/Quest_delivery.png[/img] [font_size=40]传信任务[/font_size]。</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
@@ -805,10 +797,6 @@
     <t>When you're ready,\nhead to the city gate to end the tutorial and begin your adventure.</t>
   </si>
   <si>
-    <t>Unlike [img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_new.png[/img] [font_size=40]Accepting Quests[/font_size],\n[img={"height":"35"}]res://Assets/Sprites/Icon/1x/Quest_complete.png[/img] [font_size=40]Completing Quests[/font_size] doesn't require stopping on the tile.\nPassing through will automatically deliver them.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>“Thanks for the fruit! Here are [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]Exchange Coupons x 2[/font_size].\nYou can use them at the shop.”</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -817,10 +805,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>Sometimes you'll also receive [img={"height":"40"}]res://Assets/Sprites/Icon/1x/Quest_fruit.png[/img] [font_size=40]Message Delivery Quests[/font_size],\nnot just [img={"height":"50"}]res://Assets/Sprites/Icon/1x/Quest_delivery.png[/img] [font_size=40]Fruit Quests[/font_size].</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>“Thanks for the message! Here's [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]Exchange Coupon x 1[/font_size].\nCheck out the nearby shop when you can.”</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -846,6 +830,22 @@
   </si>
   <si>
     <t>[img={"height":"45"}]res://Assets/Sprites/Icon/1x/trade_shop.png[/img] [font_size=40]The shop[/font_size] is open!\nYou can buy things with [img={"height":"50"}]res://Assets/Sprites/Icon/1x/exchange coupon italic.png[/img] [font_size=40]Exchange Coupons[/font_size].\nTake a look.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>不同于 [img={"height":"35"}]res://Assets/Sprites/Icon/1x/quest_new.png[/img] [font_size=40]接受任务[/font_size]，\n [img={"height":"35"}]res://Assets/Sprites/Icon/1x/quest_complete.png[/img] [font_size=40]完成任务 [/font_size]时不需要停留在格子上，路过就会自动交付。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>除了 [img={"height":"40"}]res://Assets/Sprites/Icon/1x/quest_fruit.png[/img] [font_size=40]水果任务[/font_size]，有时也会接到 [img={"height":"50"}]res://Assets/Sprites/Icon/1x/quest_delivery.png[/img] [font_size=40]传信任务[/font_size]。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sometimes you'll also receive [img={"height":"40"}]res://Assets/Sprites/Icon/1x/quest_fruit.png[/img] [font_size=40]Message Delivery Quests[/font_size],\nnot just [img={"height":"50"}]res://Assets/Sprites/Icon/1x/quest_delivery.png[/img] [font_size=40]Fruit Quests[/font_size].</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Unlike [img={"height":"35"}]res://Assets/Sprites/Icon/1x/quest_new.png[/img] [font_size=40]Accepting Quests[/font_size],\n[img={"height":"35"}]res://Assets/Sprites/Icon/1x/quest_complete.png[/img] [font_size=40]Completing Quests[/font_size] doesn't require stopping on the tile.\nPassing through will automatically deliver them.</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1951,7 +1951,7 @@
         <v>50</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>52</v>
@@ -2001,7 +2001,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>56</v>
@@ -2012,7 +2012,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>87</v>
@@ -2039,7 +2039,7 @@
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>85</v>
@@ -2047,10 +2047,10 @@
     </row>
     <row r="19" spans="1:3" ht="42.75">
       <c r="A19" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>88</v>
@@ -2061,7 +2061,7 @@
         <v>10</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>89</v>
@@ -2094,10 +2094,10 @@
         <v>13</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="28.5">
@@ -2105,10 +2105,10 @@
         <v>14</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -2128,7 +2128,7 @@
         <v>15</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>86</v>
@@ -2150,10 +2150,10 @@
         <v>17</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>93</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="28.5">
@@ -2161,10 +2161,10 @@
         <v>39</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2180,10 +2180,10 @@
         <v>18</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="42.75">
@@ -2191,10 +2191,10 @@
         <v>19</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="28.5">
@@ -2202,7 +2202,7 @@
         <v>20</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>59</v>
@@ -2221,10 +2221,10 @@
         <v>21</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="57">
@@ -2232,10 +2232,10 @@
         <v>22</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="42.75">
@@ -2243,10 +2243,10 @@
         <v>26</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="28.5">
@@ -2254,7 +2254,7 @@
         <v>27</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>61</v>
@@ -2265,10 +2265,10 @@
         <v>28</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
@@ -2276,10 +2276,10 @@
         <v>29</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
@@ -2287,7 +2287,7 @@
         <v>30</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>60</v>
@@ -2310,10 +2310,10 @@
         <v>40</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="28.5">
@@ -2321,10 +2321,10 @@
         <v>41</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="28.5">
@@ -2332,7 +2332,7 @@
         <v>42</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>62</v>
@@ -2376,7 +2376,7 @@
         <v>65</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>69</v>
@@ -2409,7 +2409,7 @@
         <v>31</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>82</v>

</xml_diff>